<commit_message>
Bulk import remaining 6 blog articles
Import all remaining /blog/* pages using the existing blog template + importer,
which already carries the durable fixes from the ace-pro-court-polo migration
(split columns-article parser, breadcrumb chevron, Template=blog metadata
stamping, graceful table-spec skip when a page has no spec table).

Pages: flip-flop-summer-style, latest-trends-young-casual-fashion,
fashion-trends-young-culture, fashion-trends-young-style, fashion-blog-post,
street-style-trends. All 95-96% completeness, columns-article header parsed,
template metadata stamped.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog.report.xlsx
+++ b/tools/importer/reports/import-blog.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
   <si>
     <t>_reportFile</t>
   </si>
@@ -49,7 +49,7 @@
     <t>success</t>
   </si>
   <si>
-    <t>2026-09-02T04:02:44.764Z</t>
+    <t>2026-09-02T09:28:43.805Z</t>
   </si>
   <si>
     <t>WKND Trendsetters - Fresh Looks, Bold Stories, Real Life</t>
@@ -77,6 +77,99 @@
   </si>
   <si>
     <t>https://wknd-trendsetters.site/blog/ace-pro-court-polo</t>
+  </si>
+  <si>
+    <t>blog/fashion-blog-post.report.json</t>
+  </si>
+  <si>
+    <t>["columns-article"]</t>
+  </si>
+  <si>
+    <t>blog/fashion-blog-post</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:33:14.871Z</t>
+  </si>
+  <si>
+    <t>Game on, style up | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-blog-post</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-culture.report.json</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-culture</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:33:05.631Z</t>
+  </si>
+  <si>
+    <t>Sunkissed and effortless | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-trends-young-culture</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-style.report.json</t>
+  </si>
+  <si>
+    <t>blog/fashion-trends-young-style</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:33:10.033Z</t>
+  </si>
+  <si>
+    <t>Party fits that pop | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/fashion-trends-young-style</t>
+  </si>
+  <si>
+    <t>blog/flip-flop-summer-style.report.json</t>
+  </si>
+  <si>
+    <t>blog/flip-flop-summer-style</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:32:56.858Z</t>
+  </si>
+  <si>
+    <t>Slide into summer — flip flops that serve | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/flip-flop-summer-style</t>
+  </si>
+  <si>
+    <t>blog/latest-trends-young-casual-fashion.report.json</t>
+  </si>
+  <si>
+    <t>blog/latest-trends-young-casual-fashion</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:33:01.572Z</t>
+  </si>
+  <si>
+    <t>Tennis style, redefined | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/latest-trends-young-casual-fashion</t>
+  </si>
+  <si>
+    <t>blog/street-style-trends.report.json</t>
+  </si>
+  <si>
+    <t>blog/street-style-trends</t>
+  </si>
+  <si>
+    <t>2026-09-02T17:33:19.128Z</t>
+  </si>
+  <si>
+    <t>Street style, your way | Fashion Blog</t>
+  </si>
+  <si>
+    <t>https://wknd-trendsetters.site/blog/street-style-trends</t>
   </si>
   <si>
     <t>magazine/article-1.report.json</t>
@@ -477,12 +570,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="37" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -571,25 +663,181 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
         <v>13</v>
       </c>
-      <c r="H4" t="s">
-        <v>25</v>
+      <c r="H10" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>